<commit_message>
Hyderabad book vs plant: correct the 683.8 MT note; summary sums the full range
data-verifier failed one note: only the mismatch file reads 683.8 MT; the
29-Oct ageing files read 895.2 MT (built before the 30-Sep re-upload, 2.8-3.2
kept separate). Summary figures no longer follow a filter on the size sheet;
the match count moves to the summary. Re-verification in progress.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SVVKmwQKKV189dev92iFna
</commit_message>
<xml_diff>
--- a/reports/Hyderabad-FG-Book-vs-Plant-2026-10-29.xlsx
+++ b/reports/Hyderabad-FG-Book-vs-Plant-2026-10-29.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="141">
   <si>
     <t xml:space="preserve">Hyderabad FG - book (produced minus invoiced) vs plant sheet, 29-Oct-2026</t>
   </si>
@@ -87,10 +87,16 @@
     <t xml:space="preserve">Production of 29-Oct is not yet entered in the system</t>
   </si>
   <si>
+    <t xml:space="preserve">Sizes matching within 0.5 MT (of all sizes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plant sheet FG within 0.5 MT of produced - invoiced</t>
+  </si>
+  <si>
     <t xml:space="preserve">Why this view</t>
   </si>
   <si>
-    <t xml:space="preserve">The ageing and FG files count each size at no less than 0, so a size billed beyond its production (usually made under one code and billed under a neighbouring one) cannot cancel stock held under the other code. That made the system read 683.8 MT.</t>
+    <t xml:space="preserve">The FG mismatch file counts each size at no less than 0 (2.8-3.2 as one size), so a size billed beyond its production (usually made under one code and billed under a neighbouring one) cannot cancel stock held under the other code; it read 683.8 MT. The 29-Oct ageing files read 895.2 MT for Hyderabad: they were built before the 30-Sep invoices were re-uploaded and keep 2.8-3.2 separate (720.6 MT on today's data).</t>
   </si>
   <si>
     <t xml:space="preserve">Netting every size together, as here, gives the book stock of 636.5 MT. Against the plant sheet the gap is 13.0 MT (Grand Total) or 6.9 MT (visible rows), about half a day of production: Hyderabad production for 29-Oct is not yet entered.</t>
@@ -1037,7 +1043,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="3" t="n">
-        <f aca="false">'By size'!C100</f>
+        <f aca="false">SUM('By size'!C5:C99)</f>
         <v>6960.10004706745</v>
       </c>
       <c r="C3" s="4" t="s">
@@ -1049,7 +1055,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="3" t="n">
-        <f aca="false">'By size'!E100</f>
+        <f aca="false">SUM('By size'!E5:E99)</f>
         <v>6323.554</v>
       </c>
       <c r="C4" s="4" t="s">
@@ -1084,7 +1090,7 @@
         <v>9</v>
       </c>
       <c r="B7" s="3" t="n">
-        <f aca="false">'By size'!I100</f>
+        <f aca="false">SUM('By size'!I5:I99)</f>
         <v>643.432</v>
       </c>
       <c r="C7" s="4" t="s">
@@ -1148,29 +1154,41 @@
         <v>19</v>
       </c>
     </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="3" t="str">
+        <f aca="false">COUNTIF('By size'!K5:K99,"Yes")&amp;" of "&amp;COUNTA('By size'!K5:K99)</f>
+        <v>39 of 95</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -1205,61 +1223,61 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="G4" s="11" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="H4" s="11" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="I4" s="11" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="J4" s="11" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="K4" s="11" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="L4" s="11" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="M4" s="11" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C5" s="13" t="n">
         <v>1.93886208</v>
@@ -1301,10 +1319,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C6" s="13" t="n">
         <v>22.692373056</v>
@@ -1346,10 +1364,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>43</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>41</v>
       </c>
       <c r="C7" s="13" t="n">
         <v>58.360230912</v>
@@ -1391,10 +1409,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C8" s="13" t="n">
         <v>71.5068432</v>
@@ -1436,10 +1454,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C9" s="13" t="n">
         <v>24.735096288</v>
@@ -1481,10 +1499,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C10" s="13" t="n">
         <v>145.722305664</v>
@@ -1526,10 +1544,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C11" s="13" t="n">
         <v>213.7047576</v>
@@ -1571,10 +1589,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C12" s="13" t="n">
         <v>80.41383</v>
@@ -1616,10 +1634,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C13" s="13" t="n">
         <v>41.907798848</v>
@@ -1661,10 +1679,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C14" s="13" t="n">
         <v>51.861907968</v>
@@ -1706,10 +1724,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="12" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C15" s="13" t="n">
         <v>40.0176672</v>
@@ -1751,10 +1769,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C16" s="13" t="n">
         <v>30.1145625</v>
@@ -1796,10 +1814,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="12" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C17" s="13" t="n">
         <v>180.99000192</v>
@@ -1841,10 +1859,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="12" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C18" s="13" t="n">
         <v>229.380768</v>
@@ -1886,10 +1904,10 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="12" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C19" s="13" t="n">
         <v>16.233192096</v>
@@ -1931,10 +1949,10 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="12" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C20" s="13" t="n">
         <v>149.748798</v>
@@ -1976,10 +1994,10 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="12" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C21" s="13" t="n">
         <v>93.382012416</v>
@@ -2021,10 +2039,10 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="12" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C22" s="13" t="n">
         <v>16.592</v>
@@ -2066,10 +2084,10 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C23" s="13" t="n">
         <v>32.998817664</v>
@@ -2111,10 +2129,10 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C24" s="13" t="n">
         <v>155.555338752</v>
@@ -2156,10 +2174,10 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="12" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C25" s="13" t="n">
         <v>362.0354688</v>
@@ -2201,10 +2219,10 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C26" s="13" t="n">
         <v>8.578658352</v>
@@ -2246,10 +2264,10 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="12" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C27" s="13" t="n">
         <v>159.0461025</v>
@@ -2291,10 +2309,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="12" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C28" s="13" t="n">
         <v>187.846902816</v>
@@ -2336,10 +2354,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="12" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C29" s="13" t="n">
         <v>76.4723136</v>
@@ -2381,10 +2399,10 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="12" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C30" s="13" t="n">
         <v>49.918</v>
@@ -2426,10 +2444,10 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="12" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C31" s="13" t="n">
         <v>28.9511925</v>
@@ -2471,10 +2489,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C32" s="13" t="n">
         <v>31.38110976</v>
@@ -2516,10 +2534,10 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C33" s="13" t="n">
         <v>28.9502976</v>
@@ -2561,10 +2579,10 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="12" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C34" s="13" t="n">
         <v>25.3</v>
@@ -2606,10 +2624,10 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="12" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C35" s="13" t="n">
         <v>25.875</v>
@@ -2651,10 +2669,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="12" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C36" s="13" t="n">
         <v>20.24953344</v>
@@ -2696,10 +2714,10 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="12" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C37" s="13" t="n">
         <v>52.700875776</v>
@@ -2741,10 +2759,10 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="B38" s="2" t="s">
         <v>75</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>73</v>
       </c>
       <c r="C38" s="13" t="n">
         <v>116.5397184</v>
@@ -2786,10 +2804,10 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="12" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C39" s="13" t="n">
         <v>2.47734696</v>
@@ -2831,10 +2849,10 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="12" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C40" s="13" t="n">
         <v>24.0786975</v>
@@ -2876,10 +2894,10 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="12" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C41" s="13" t="n">
         <v>26.010473856</v>
@@ -2921,10 +2939,10 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="12" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C42" s="13" t="n">
         <v>100.544377536</v>
@@ -2966,10 +2984,10 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="12" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C43" s="13" t="n">
         <v>96.0559284</v>
@@ -3011,10 +3029,10 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="12" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C44" s="13" t="n">
         <v>59.87352</v>
@@ -3056,10 +3074,10 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="12" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C45" s="13" t="n">
         <v>37.927843968</v>
@@ -3101,10 +3119,10 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="12" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C46" s="13" t="n">
         <v>215.373092352</v>
@@ -3146,10 +3164,10 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="12" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C47" s="13" t="n">
         <v>292.2219648</v>
@@ -3191,10 +3209,10 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="12" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C48" s="13" t="n">
         <v>126.6954675</v>
@@ -3236,10 +3254,10 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="12" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C49" s="13" t="n">
         <v>93.595130496</v>
@@ -3281,10 +3299,10 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="12" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C50" s="13" t="n">
         <v>74.290732032</v>
@@ -3326,10 +3344,10 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="12" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C51" s="13" t="n">
         <v>73.7563392</v>
@@ -3371,10 +3389,10 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="12" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C52" s="13" t="n">
         <v>17.405805</v>
@@ -3416,10 +3434,10 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="12" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C53" s="13" t="n">
         <v>27.26434368</v>
@@ -3461,10 +3479,10 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="12" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C54" s="13" t="n">
         <v>126.326992896</v>
@@ -3506,10 +3524,10 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="12" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C55" s="13" t="n">
         <v>271.4097936</v>
@@ -3551,10 +3569,10 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="12" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C56" s="13" t="n">
         <v>133.950045</v>
@@ -3596,10 +3614,10 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="12" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C57" s="13" t="n">
         <v>139.776190656</v>
@@ -3641,10 +3659,10 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="12" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C58" s="13" t="n">
         <v>69.8014464</v>
@@ -3686,10 +3704,10 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="12" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C59" s="13" t="n">
         <v>90.007331328</v>
@@ -3731,10 +3749,10 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="12" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C60" s="13" t="n">
         <v>225.6349992</v>
@@ -3776,10 +3794,10 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="12" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C61" s="13" t="n">
         <v>96.1935075</v>
@@ -3821,10 +3839,10 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="12" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C62" s="13" t="n">
         <v>134.376193248</v>
@@ -3866,10 +3884,10 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="12" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C63" s="13" t="n">
         <v>100.9650672</v>
@@ -3911,10 +3929,10 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="12" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C64" s="13" t="n">
         <v>28.4829461399923</v>
@@ -3956,10 +3974,10 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="12" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C65" s="13" t="n">
         <v>39.2502</v>
@@ -4001,10 +4019,10 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="12" t="s">
+        <v>106</v>
+      </c>
+      <c r="B66" s="2" t="s">
         <v>104</v>
-      </c>
-      <c r="B66" s="2" t="s">
-        <v>102</v>
       </c>
       <c r="C66" s="13" t="n">
         <v>5.2602</v>
@@ -4044,10 +4062,10 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="12" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C67" s="13" t="n">
         <v>56.9928108030086</v>
@@ -4089,10 +4107,10 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="12" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C68" s="13" t="n">
         <v>84.3734114638618</v>
@@ -4134,10 +4152,10 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="12" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C69" s="13" t="n">
         <v>24.9481676337717</v>
@@ -4179,10 +4197,10 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="12" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C70" s="13" t="n">
         <v>25.9109428201605</v>
@@ -4224,10 +4242,10 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="12" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C71" s="13" t="n">
         <v>47.5740503744717</v>
@@ -4269,10 +4287,10 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="12" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C72" s="13" t="n">
         <v>56.1091694452986</v>
@@ -4314,10 +4332,10 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="12" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C73" s="13" t="n">
         <v>28.4615439018097</v>
@@ -4359,10 +4377,10 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="12" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B74" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C74" s="13" t="n">
         <v>27.54</v>
@@ -4404,10 +4422,10 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="12" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C75" s="13" t="n">
         <v>4.576</v>
@@ -4449,10 +4467,10 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="12" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C76" s="13" t="n">
         <v>26.5054408870247</v>
@@ -4494,10 +4512,10 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="12" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C77" s="13" t="n">
         <v>72.1179666620389</v>
@@ -4539,10 +4557,10 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="12" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C78" s="13" t="n">
         <v>57.4455663919972</v>
@@ -4584,10 +4602,10 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="12" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C79" s="13" t="n">
         <v>63.5927733526701</v>
@@ -4629,10 +4647,10 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="12" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C80" s="13" t="n">
         <v>9.79578547616842</v>
@@ -4674,10 +4692,10 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="12" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B81" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C81" s="13" t="n">
         <v>36.3308201659899</v>
@@ -4719,10 +4737,10 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="12" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C82" s="13" t="n">
         <v>84.1161525361491</v>
@@ -4764,10 +4782,10 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="12" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C83" s="13" t="n">
         <v>28.3616648173704</v>
@@ -4809,10 +4827,10 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="12" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C84" s="13" t="n">
         <v>83.9631429770518</v>
@@ -4854,10 +4872,10 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="12" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C85" s="13" t="n">
         <v>35.133</v>
@@ -4899,10 +4917,10 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="12" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C86" s="13" t="n">
         <v>41.9696943760219</v>
@@ -4944,10 +4962,10 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="12" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B87" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C87" s="13" t="n">
         <v>51.8458270267837</v>
@@ -4989,10 +5007,10 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="12" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C88" s="13" t="n">
         <v>28.0525575471577</v>
@@ -5034,10 +5052,10 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="12" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C89" s="13" t="n">
         <v>99.9575553667495</v>
@@ -5079,10 +5097,10 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="12" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C90" s="13" t="n">
         <v>6.74887264657441</v>
@@ -5124,10 +5142,10 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="12" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C91" s="13" t="n">
         <v>38.2222607216639</v>
@@ -5169,10 +5187,10 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="12" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C92" s="13" t="n">
         <v>20.5286291240952</v>
@@ -5214,10 +5232,10 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="12" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B93" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C93" s="13" t="n">
         <v>47.6188435543849</v>
@@ -5259,10 +5277,10 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="12" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C94" s="13" t="n">
         <v>12.4272</v>
@@ -5304,10 +5322,10 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="12" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C95" s="13" t="n">
         <v>18.45</v>
@@ -5349,10 +5367,10 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="12" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B96" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C96" s="13" t="n">
         <v>30.4489453224326</v>
@@ -5394,10 +5412,10 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="12" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C97" s="13" t="n">
         <v>54.0465701717689</v>
@@ -5439,10 +5457,10 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="12" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C98" s="13" t="n">
         <v>58.1552673449761</v>
@@ -5484,10 +5502,10 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="12" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C99" s="13" t="n">
         <v>37.0711</v>
@@ -5529,7 +5547,7 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B100" s="5"/>
       <c r="C100" s="19" t="n">
@@ -5564,10 +5582,7 @@
         <f aca="false">SUBTOTAL(9,J5:J99)</f>
         <v>6.88595293255524</v>
       </c>
-      <c r="K100" s="5" t="str">
-        <f aca="false">COUNTIF(K5:K99,"Yes")&amp;" of "&amp;COUNTA(K5:K99)&amp;" match"</f>
-        <v>39 of 95 match</v>
-      </c>
+      <c r="K100" s="5"/>
       <c r="L100" s="5"/>
       <c r="M100" s="5"/>
     </row>

</xml_diff>